<commit_message>
Continue to review code
Deterministic, uncertainty and robust problem cells
</commit_message>
<xml_diff>
--- a/Project/Project_database.xlsx
+++ b/Project/Project_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Robust Optimization/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="316" documentId="13_ncr:1_{3569C1BF-E599-4CC3-958C-CF2B068FF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6657BEB7-4EA0-4962-A8DB-DEF02DBF2456}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="13_ncr:1_{3569C1BF-E599-4CC3-958C-CF2B068FF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{808C090E-6786-43A3-A2D5-67C545127A7F}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{66A798E0-9E9A-4626-9FF9-44F67D5440CA}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66A798E0-9E9A-4626-9FF9-44F67D5440CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Item characteristics" sheetId="1" r:id="rId1"/>
@@ -2053,6 +2053,8 @@
       <c r="M18" s="1"/>
       <c r="O18" s="1"/>
       <c r="Q18" s="4"/>
+      <c r="AB18" s="1"/>
+      <c r="AC18" s="1"/>
     </row>
     <row r="19" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F19" s="1"/>
@@ -2060,6 +2062,8 @@
       <c r="M19" s="1"/>
       <c r="O19" s="1"/>
       <c r="Q19" s="4"/>
+      <c r="AB19" s="1"/>
+      <c r="AC19" s="1"/>
     </row>
     <row r="20" spans="3:29" x14ac:dyDescent="0.25">
       <c r="C20" s="4"/>
@@ -2074,6 +2078,8 @@
       <c r="M20" s="1"/>
       <c r="O20" s="1"/>
       <c r="Q20" s="4"/>
+      <c r="AB20" s="1"/>
+      <c r="AC20" s="1"/>
     </row>
     <row r="21" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F21" s="4"/>
@@ -2083,7 +2089,8 @@
       <c r="O21" s="1"/>
       <c r="Q21" s="4"/>
       <c r="S21" s="3"/>
-      <c r="AC21" s="4"/>
+      <c r="AB21" s="1"/>
+      <c r="AC21" s="1"/>
     </row>
     <row r="22" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F22" s="1"/>
@@ -2093,7 +2100,8 @@
       <c r="O22" s="1"/>
       <c r="Q22" s="4"/>
       <c r="S22" s="3"/>
-      <c r="AC22" s="4"/>
+      <c r="AB22" s="1"/>
+      <c r="AC22" s="1"/>
     </row>
     <row r="23" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F23" s="2"/>
@@ -2102,7 +2110,8 @@
       <c r="O23" s="1"/>
       <c r="Q23" s="4"/>
       <c r="S23" s="3"/>
-      <c r="AC23" s="4"/>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="1"/>
     </row>
     <row r="24" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F24" s="1"/>
@@ -2111,7 +2120,8 @@
       <c r="O24" s="1"/>
       <c r="Q24" s="4"/>
       <c r="S24" s="3"/>
-      <c r="AC24" s="4"/>
+      <c r="AB24" s="1"/>
+      <c r="AC24" s="1"/>
     </row>
     <row r="25" spans="3:29" x14ac:dyDescent="0.25">
       <c r="F25" s="1"/>

</xml_diff>

<commit_message>
Final commit for user manuals
</commit_message>
<xml_diff>
--- a/Project/Project_database.xlsx
+++ b/Project/Project_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Robust Optimization/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="13_ncr:1_{3569C1BF-E599-4CC3-958C-CF2B068FF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{808C090E-6786-43A3-A2D5-67C545127A7F}"/>
+  <xr:revisionPtr revIDLastSave="327" documentId="13_ncr:1_{3569C1BF-E599-4CC3-958C-CF2B068FF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44E8F058-A85D-452F-A1F2-C456DA3645AD}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66A798E0-9E9A-4626-9FF9-44F67D5440CA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66A798E0-9E9A-4626-9FF9-44F67D5440CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Item characteristics" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="79">
   <si>
     <t>a</t>
   </si>
@@ -195,24 +195,6 @@
   </si>
   <si>
     <t>BMPinf Min</t>
-  </si>
-  <si>
-    <t>TS Max/Mean</t>
-  </si>
-  <si>
-    <t>TS Min/Mean</t>
-  </si>
-  <si>
-    <t>VS Max/Mean</t>
-  </si>
-  <si>
-    <t>VS Min/Mean</t>
-  </si>
-  <si>
-    <t>BMP Max/Mean</t>
-  </si>
-  <si>
-    <t>BMP Min/Mean</t>
   </si>
   <si>
     <t>kgFM/m3FM</t>
@@ -750,36 +732,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587CCA70-3B8D-4DF4-BACF-B592D887B522}">
-  <dimension ref="A1:AD36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X36"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>30</v>
@@ -848,104 +825,80 @@
         <v>51</v>
       </c>
       <c r="X1" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y1" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z1" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="AA1" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="AB1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="AC1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="AD1" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
       <c r="B2" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="I2" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="K2" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="L2" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="M2" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="N2" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="I2" s="14" t="s">
+      <c r="O2" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L2" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="M2" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="N2" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="O2" s="14" t="s">
-        <v>69</v>
-      </c>
       <c r="P2" s="14" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="Q2" s="14" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="R2" s="14" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="S2" s="14" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="T2" s="14" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="U2" s="14" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="V2" s="14" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="W2" s="14" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14"/>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
-      <c r="AD2" s="14"/>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
@@ -1018,35 +971,11 @@
       <c r="W3" s="17">
         <v>286.2</v>
       </c>
-      <c r="X3" s="15">
-        <f t="shared" ref="X3:X12" si="0">R3/C3</f>
-        <v>0.8571428571428571</v>
-      </c>
-      <c r="Y3" s="15">
-        <f t="shared" ref="Y3:Y12" si="1">S3/C3</f>
-        <v>1.1428571428571428</v>
-      </c>
-      <c r="Z3" s="15">
-        <f t="shared" ref="Z3:Z12" si="2">T3/D3</f>
-        <v>0.83971948368736671</v>
-      </c>
-      <c r="AA3" s="15">
-        <f t="shared" ref="AA3:AA12" si="3">U3/D3</f>
-        <v>1.1464579733712776</v>
-      </c>
-      <c r="AB3" s="15">
-        <f t="shared" ref="AB3:AB12" si="4">V3/E3</f>
-        <v>1.0491996342789045</v>
-      </c>
-      <c r="AC3" s="15">
-        <f t="shared" ref="AC3:AC12" si="5">W3/E3</f>
-        <v>0.92682447654279154</v>
-      </c>
-      <c r="AD3" s="14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X3" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>21</v>
       </c>
@@ -1097,7 +1026,7 @@
         <v>100</v>
       </c>
       <c r="Q4" s="17">
-        <f t="shared" ref="Q4:Q12" si="6">E4-P4</f>
+        <f t="shared" ref="Q4:Q12" si="0">E4-P4</f>
         <v>194.36180555555558</v>
       </c>
       <c r="R4" s="17">
@@ -1118,35 +1047,11 @@
       <c r="W4" s="17">
         <v>185.7</v>
       </c>
-      <c r="X4" s="15">
-        <f t="shared" si="0"/>
-        <v>0.61128697740421345</v>
-      </c>
-      <c r="Y4" s="15">
-        <f t="shared" si="1"/>
-        <v>1.4867372557581049</v>
-      </c>
-      <c r="Z4" s="15">
-        <f t="shared" si="2"/>
-        <v>0.62602474288269494</v>
-      </c>
-      <c r="AA4" s="15">
-        <f t="shared" si="3"/>
-        <v>1.4398569086301982</v>
-      </c>
-      <c r="AB4" s="15">
-        <f t="shared" si="4"/>
-        <v>1.27394245082936</v>
-      </c>
-      <c r="AC4" s="15">
-        <f t="shared" si="5"/>
-        <v>0.63085630165069906</v>
-      </c>
-      <c r="AD4" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X4" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>22</v>
       </c>
@@ -1197,7 +1102,7 @@
         <v>50</v>
       </c>
       <c r="Q5" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>132.1875</v>
       </c>
       <c r="R5" s="17">
@@ -1218,35 +1123,11 @@
       <c r="W5" s="17">
         <v>165</v>
       </c>
-      <c r="X5" s="15">
-        <f t="shared" si="0"/>
-        <v>0.90721649484536082</v>
-      </c>
-      <c r="Y5" s="15">
-        <f t="shared" si="1"/>
-        <v>1.0309278350515463</v>
-      </c>
-      <c r="Z5" s="15">
-        <f t="shared" si="2"/>
-        <v>0.88958009331259713</v>
-      </c>
-      <c r="AA5" s="15">
-        <f t="shared" si="3"/>
-        <v>1.0368066355624677</v>
-      </c>
-      <c r="AB5" s="15">
-        <f t="shared" si="4"/>
-        <v>1.1471698113207549</v>
-      </c>
-      <c r="AC5" s="15">
-        <f t="shared" si="5"/>
-        <v>0.90566037735849059</v>
-      </c>
-      <c r="AD5" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X5" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>23</v>
       </c>
@@ -1298,7 +1179,7 @@
         <v>50</v>
       </c>
       <c r="Q6" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>181.35999999999999</v>
       </c>
       <c r="R6" s="17">
@@ -1319,35 +1200,11 @@
       <c r="W6" s="17">
         <v>181.5</v>
       </c>
-      <c r="X6" s="15">
-        <f t="shared" si="0"/>
-        <v>0.18248632396542361</v>
-      </c>
-      <c r="Y6" s="15">
-        <f t="shared" si="1"/>
-        <v>2.0225219582132765</v>
-      </c>
-      <c r="Z6" s="15">
-        <f t="shared" si="2"/>
-        <v>9.3913973463453759E-2</v>
-      </c>
-      <c r="AA6" s="15">
-        <f t="shared" si="3"/>
-        <v>2.0737943250559807</v>
-      </c>
-      <c r="AB6" s="15">
-        <f t="shared" si="4"/>
-        <v>1.3831258644536655</v>
-      </c>
-      <c r="AC6" s="15">
-        <f t="shared" si="5"/>
-        <v>0.78449170124481338</v>
-      </c>
-      <c r="AD6" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X6" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>24</v>
       </c>
@@ -1399,7 +1256,7 @@
         <v>200</v>
       </c>
       <c r="Q7" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>143.74585454545456</v>
       </c>
       <c r="R7" s="17">
@@ -1420,35 +1277,11 @@
       <c r="W7" s="17">
         <v>295.06440000000003</v>
       </c>
-      <c r="X7" s="15">
-        <f t="shared" si="0"/>
-        <v>0.67639331432724026</v>
-      </c>
-      <c r="Y7" s="15">
-        <f t="shared" si="1"/>
-        <v>1.1424897982000113</v>
-      </c>
-      <c r="Z7" s="15">
-        <f t="shared" si="2"/>
-        <v>0.67575018743616833</v>
-      </c>
-      <c r="AA7" s="15">
-        <f t="shared" si="3"/>
-        <v>1.1890242102591047</v>
-      </c>
-      <c r="AB7" s="15">
-        <f t="shared" si="4"/>
-        <v>1.1636503966831309</v>
-      </c>
-      <c r="AC7" s="15">
-        <f t="shared" si="5"/>
-        <v>0.85837951526767509</v>
-      </c>
-      <c r="AD7" s="14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X7" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -1499,7 +1332,7 @@
         <v>70</v>
       </c>
       <c r="Q8" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>132.32</v>
       </c>
       <c r="R8" s="17">
@@ -1520,35 +1353,11 @@
       <c r="W8" s="17">
         <v>125</v>
       </c>
-      <c r="X8" s="15">
-        <f t="shared" si="0"/>
-        <v>0.68252730109204374</v>
-      </c>
-      <c r="Y8" s="15">
-        <f t="shared" si="1"/>
-        <v>1.3299531981279253</v>
-      </c>
-      <c r="Z8" s="15">
-        <f t="shared" si="2"/>
-        <v>0.70778564206268957</v>
-      </c>
-      <c r="AA8" s="15">
-        <f t="shared" si="3"/>
-        <v>1.236097067745197</v>
-      </c>
-      <c r="AB8" s="15">
-        <f t="shared" si="4"/>
-        <v>1.2470344009489918</v>
-      </c>
-      <c r="AC8" s="15">
-        <f t="shared" si="5"/>
-        <v>0.61783313562672992</v>
-      </c>
-      <c r="AD8" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X8" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>26</v>
       </c>
@@ -1600,7 +1409,7 @@
         <v>120</v>
       </c>
       <c r="Q9" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>160.4325</v>
       </c>
       <c r="R9" s="17">
@@ -1621,35 +1430,11 @@
       <c r="W9" s="17">
         <v>152</v>
       </c>
-      <c r="X9" s="15">
-        <f t="shared" si="0"/>
-        <v>0.70750930806053869</v>
-      </c>
-      <c r="Y9" s="15">
-        <f t="shared" si="1"/>
-        <v>1.237851167738504</v>
-      </c>
-      <c r="Z9" s="15">
-        <f t="shared" si="2"/>
-        <v>0.7092584834520318</v>
-      </c>
-      <c r="AA9" s="15">
-        <f t="shared" si="3"/>
-        <v>1.2601591956430662</v>
-      </c>
-      <c r="AB9" s="15">
-        <f t="shared" si="4"/>
-        <v>1.329945708860421</v>
-      </c>
-      <c r="AC9" s="15">
-        <f t="shared" si="5"/>
-        <v>0.54201991566598018</v>
-      </c>
-      <c r="AD9" s="14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X9" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>27</v>
       </c>
@@ -1700,7 +1485,7 @@
         <v>30</v>
       </c>
       <c r="Q10" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>161.375</v>
       </c>
       <c r="R10" s="17">
@@ -1721,35 +1506,11 @@
       <c r="W10" s="17">
         <v>170</v>
       </c>
-      <c r="X10" s="15">
-        <f t="shared" si="0"/>
-        <v>0.97777777777777775</v>
-      </c>
-      <c r="Y10" s="15">
-        <f t="shared" si="1"/>
-        <v>1.016888888888889</v>
-      </c>
-      <c r="Z10" s="15">
-        <f t="shared" si="2"/>
-        <v>0.97777777777777775</v>
-      </c>
-      <c r="AA10" s="15">
-        <f t="shared" si="3"/>
-        <v>1.016888888888889</v>
-      </c>
-      <c r="AB10" s="15">
-        <f t="shared" si="4"/>
-        <v>1.1652514696276943</v>
-      </c>
-      <c r="AC10" s="15">
-        <f t="shared" si="5"/>
-        <v>0.8883082952318746</v>
-      </c>
-      <c r="AD10" s="14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X10" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>28</v>
       </c>
@@ -1801,7 +1562,7 @@
         <v>120</v>
       </c>
       <c r="Q11" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>168.5</v>
       </c>
       <c r="R11" s="17">
@@ -1822,35 +1583,11 @@
       <c r="W11" s="17">
         <v>238</v>
       </c>
-      <c r="X11" s="15">
-        <f t="shared" si="0"/>
-        <v>0.93333333333333335</v>
-      </c>
-      <c r="Y11" s="15">
-        <f t="shared" si="1"/>
-        <v>1.0666666666666667</v>
-      </c>
-      <c r="Z11" s="15">
-        <f t="shared" si="2"/>
-        <v>0.93843711412947617</v>
-      </c>
-      <c r="AA11" s="15">
-        <f t="shared" si="3"/>
-        <v>1.0612100899629564</v>
-      </c>
-      <c r="AB11" s="15">
-        <f t="shared" si="4"/>
-        <v>1.2166377816291161</v>
-      </c>
-      <c r="AC11" s="15">
-        <f t="shared" si="5"/>
-        <v>0.82495667244367421</v>
-      </c>
-      <c r="AD11" s="14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X11" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>29</v>
       </c>
@@ -1901,7 +1638,7 @@
         <v>70</v>
       </c>
       <c r="Q12" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="0"/>
         <v>261.88416666666672</v>
       </c>
       <c r="R12" s="17">
@@ -1922,49 +1659,19 @@
       <c r="W12" s="17">
         <v>304.2</v>
       </c>
-      <c r="X12" s="15">
-        <f t="shared" si="0"/>
-        <v>0.98360655737704916</v>
-      </c>
-      <c r="Y12" s="15">
-        <f t="shared" si="1"/>
-        <v>1.0175240248728095</v>
-      </c>
-      <c r="Z12" s="15">
-        <f t="shared" si="2"/>
-        <v>0.92421297535712199</v>
-      </c>
-      <c r="AA12" s="15">
-        <f t="shared" si="3"/>
-        <v>1.0480456290014515</v>
-      </c>
-      <c r="AB12" s="15">
-        <f t="shared" si="4"/>
-        <v>1.1061088080429666</v>
-      </c>
-      <c r="AC12" s="15">
-        <f t="shared" si="5"/>
-        <v>0.91658485264688216</v>
-      </c>
-      <c r="AD12" s="14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X12" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="J13" s="6"/>
       <c r="O13" s="5"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="1"/>
-      <c r="Z13" s="1"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="1"/>
-      <c r="AC13" s="1"/>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -1979,14 +1686,8 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="1"/>
-      <c r="Y14" s="1"/>
-      <c r="Z14" s="1"/>
-      <c r="AA14" s="1"/>
-      <c r="AB14" s="1"/>
-      <c r="AC14" s="1"/>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -2001,14 +1702,8 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="W15" s="1"/>
-      <c r="X15" s="1"/>
-      <c r="Y15" s="1"/>
-      <c r="Z15" s="1"/>
-      <c r="AA15" s="1"/>
-      <c r="AB15" s="1"/>
-      <c r="AC15" s="1"/>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="F16" s="3"/>
@@ -2024,14 +1719,8 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="W16" s="1"/>
-      <c r="X16" s="1"/>
-      <c r="Y16" s="1"/>
-      <c r="Z16" s="1"/>
-      <c r="AA16" s="1"/>
-      <c r="AB16" s="1"/>
-      <c r="AC16" s="1"/>
-    </row>
-    <row r="17" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="M17" s="1"/>
@@ -2040,32 +1729,22 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
       <c r="W17" s="1"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="1"/>
-      <c r="Z17" s="1"/>
-      <c r="AA17" s="1"/>
-      <c r="AB17" s="1"/>
-      <c r="AC17" s="1"/>
-    </row>
-    <row r="18" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="M18" s="1"/>
       <c r="O18" s="1"/>
       <c r="Q18" s="4"/>
-      <c r="AB18" s="1"/>
-      <c r="AC18" s="1"/>
-    </row>
-    <row r="19" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="M19" s="1"/>
       <c r="O19" s="1"/>
       <c r="Q19" s="4"/>
-      <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
-    </row>
-    <row r="20" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="F20" s="4"/>
@@ -2078,10 +1757,8 @@
       <c r="M20" s="1"/>
       <c r="O20" s="1"/>
       <c r="Q20" s="4"/>
-      <c r="AB20" s="1"/>
-      <c r="AC20" s="1"/>
-    </row>
-    <row r="21" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="M21" s="1"/>
@@ -2089,10 +1766,8 @@
       <c r="O21" s="1"/>
       <c r="Q21" s="4"/>
       <c r="S21" s="3"/>
-      <c r="AB21" s="1"/>
-      <c r="AC21" s="1"/>
-    </row>
-    <row r="22" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="M22" s="1"/>
@@ -2100,88 +1775,70 @@
       <c r="O22" s="1"/>
       <c r="Q22" s="4"/>
       <c r="S22" s="3"/>
-      <c r="AB22" s="1"/>
-      <c r="AC22" s="1"/>
-    </row>
-    <row r="23" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="M23" s="1"/>
       <c r="O23" s="1"/>
       <c r="Q23" s="4"/>
       <c r="S23" s="3"/>
-      <c r="AB23" s="1"/>
-      <c r="AC23" s="1"/>
-    </row>
-    <row r="24" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="M24" s="1"/>
       <c r="O24" s="1"/>
       <c r="Q24" s="4"/>
       <c r="S24" s="3"/>
-      <c r="AB24" s="1"/>
-      <c r="AC24" s="1"/>
-    </row>
-    <row r="25" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="M25" s="1"/>
       <c r="O25" s="1"/>
       <c r="Q25" s="4"/>
       <c r="S25" s="3"/>
-      <c r="AC25" s="4"/>
-    </row>
-    <row r="26" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="M26" s="1"/>
       <c r="Q26" s="4"/>
       <c r="S26" s="3"/>
-      <c r="AC26" s="4"/>
-    </row>
-    <row r="27" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="M27" s="1"/>
       <c r="Q27" s="4"/>
       <c r="S27" s="3"/>
-      <c r="AC27" s="4"/>
-    </row>
-    <row r="28" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="M28" s="1"/>
       <c r="S28" s="3"/>
-      <c r="AC28" s="4"/>
-    </row>
-    <row r="29" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="S29" s="3"/>
-      <c r="AC29" s="4"/>
-    </row>
-    <row r="30" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="S30" s="3"/>
-      <c r="AC30" s="4"/>
-    </row>
-    <row r="31" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
-      <c r="X31" s="1"/>
-      <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-      <c r="AA31" s="1"/>
-      <c r="AB31" s="1"/>
-      <c r="AC31" s="1"/>
-    </row>
-    <row r="32" spans="3:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
@@ -2196,60 +1853,30 @@
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
-      <c r="X32" s="1"/>
-      <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-      <c r="AA32" s="1"/>
-      <c r="AB32" s="1"/>
-      <c r="AC32" s="1"/>
-    </row>
-    <row r="33" spans="20:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
-      <c r="X33" s="1"/>
-      <c r="Y33" s="1"/>
-      <c r="Z33" s="1"/>
-      <c r="AA33" s="1"/>
-      <c r="AB33" s="1"/>
-      <c r="AC33" s="1"/>
-    </row>
-    <row r="34" spans="20:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T34" s="1"/>
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
-      <c r="X34" s="1"/>
-      <c r="Y34" s="1"/>
-      <c r="Z34" s="1"/>
-      <c r="AA34" s="1"/>
-      <c r="AB34" s="1"/>
-      <c r="AC34" s="1"/>
-    </row>
-    <row r="35" spans="20:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
-      <c r="X35" s="1"/>
-      <c r="Y35" s="1"/>
-      <c r="Z35" s="1"/>
-      <c r="AA35" s="1"/>
-      <c r="AB35" s="1"/>
-      <c r="AC35" s="1"/>
-    </row>
-    <row r="36" spans="20:29" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
-      <c r="X36" s="1"/>
-      <c r="Y36" s="1"/>
-      <c r="Z36" s="1"/>
-      <c r="AA36" s="1"/>
-      <c r="AB36" s="1"/>
-      <c r="AC36" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2259,26 +1886,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DA4D964-1DBF-442F-96AD-DD78914AF189}">
   <dimension ref="A1:W52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
       <c r="B2" s="14" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>0</v>
       </c>
@@ -2286,7 +1913,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
@@ -2294,7 +1921,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>2</v>
       </c>
@@ -2302,7 +1929,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>3</v>
       </c>
@@ -2310,7 +1937,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>4</v>
       </c>
@@ -2318,7 +1945,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>5</v>
       </c>
@@ -2326,7 +1953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>6</v>
       </c>
@@ -2334,7 +1961,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>7</v>
       </c>
@@ -2342,7 +1969,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>8</v>
       </c>
@@ -2350,7 +1977,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>9</v>
       </c>
@@ -2358,7 +1985,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>10</v>
       </c>
@@ -2366,7 +1993,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>11</v>
       </c>
@@ -2374,7 +2001,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>12</v>
       </c>
@@ -2382,7 +2009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>13</v>
       </c>
@@ -2390,7 +2017,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>14</v>
       </c>
@@ -2398,7 +2025,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>15</v>
       </c>
@@ -2406,7 +2033,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>16</v>
       </c>
@@ -2414,7 +2041,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>17</v>
       </c>
@@ -2422,7 +2049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
         <v>18</v>
       </c>
@@ -2430,7 +2057,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>19</v>
       </c>
@@ -2438,7 +2065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
@@ -2450,37 +2077,37 @@
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
     </row>
-    <row r="33" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W33" s="6"/>
     </row>
-    <row r="34" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W34" s="6"/>
     </row>
-    <row r="35" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W35" s="6"/>
     </row>
-    <row r="36" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W36" s="6"/>
     </row>
-    <row r="37" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W37" s="6"/>
     </row>
-    <row r="38" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W38" s="6"/>
     </row>
-    <row r="39" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W39" s="6"/>
     </row>
-    <row r="40" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W40" s="6"/>
     </row>
-    <row r="41" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W41" s="6"/>
     </row>
-    <row r="42" spans="23:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="23:23" x14ac:dyDescent="0.3">
       <c r="W42" s="6"/>
     </row>
-    <row r="52" spans="4:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -2500,19 +2127,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6DFE855-BBB5-4219-BB51-343CE96B9B49}">
   <dimension ref="A1:M49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>20</v>
@@ -2545,42 +2172,42 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="16"/>
       <c r="B2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="K2" s="14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B3" s="17">
         <v>7923.5999999999913</v>
@@ -2614,9 +2241,9 @@
         <v>21160.041000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B4" s="17">
         <v>8555.5555555555457</v>
@@ -2650,9 +2277,9 @@
         <v>27828.368750000001</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B5" s="17">
         <v>7247.3333333333258</v>
@@ -2686,9 +2313,9 @@
         <v>17293.237499999999</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B6" s="15">
         <f>B4/B3</f>
@@ -2731,9 +2358,9 @@
         <v>1.3151377518597434</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B7" s="15">
         <f>B5/B3</f>
@@ -2776,7 +2403,7 @@
         <v>0.81725916788157427</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>0</v>
       </c>
@@ -2811,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>1</v>
       </c>
@@ -2846,7 +2473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>2</v>
       </c>
@@ -2881,7 +2508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>3</v>
       </c>
@@ -2916,7 +2543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>4</v>
       </c>
@@ -2951,7 +2578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>5</v>
       </c>
@@ -2987,7 +2614,7 @@
       </c>
       <c r="M13" s="21"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>6</v>
       </c>
@@ -3022,7 +2649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>7</v>
       </c>
@@ -3057,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>8</v>
       </c>
@@ -3092,7 +2719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>9</v>
       </c>
@@ -3127,7 +2754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>10</v>
       </c>
@@ -3162,7 +2789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>11</v>
       </c>
@@ -3197,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>12</v>
       </c>
@@ -3232,7 +2859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
         <v>13</v>
       </c>
@@ -3267,7 +2894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>14</v>
       </c>
@@ -3302,7 +2929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
         <v>15</v>
       </c>
@@ -3337,7 +2964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
         <v>16</v>
       </c>
@@ -3372,7 +2999,7 @@
         <v>14834.97014602643</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
         <v>17</v>
       </c>
@@ -3407,7 +3034,7 @@
         <v>6229.9622564825358</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
         <v>18</v>
       </c>
@@ -3442,7 +3069,7 @@
         <v>95.108597491038353</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
         <v>19</v>
       </c>
@@ -3477,10 +3104,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -3492,7 +3119,7 @@
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -3504,7 +3131,7 @@
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -3516,7 +3143,7 @@
       <c r="J32" s="17"/>
       <c r="K32" s="17"/>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B33" s="17"/>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
@@ -3528,7 +3155,7 @@
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -3540,7 +3167,7 @@
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -3552,7 +3179,7 @@
       <c r="J35" s="17"/>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -3564,7 +3191,7 @@
       <c r="J36" s="17"/>
       <c r="K36" s="17"/>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -3576,7 +3203,7 @@
       <c r="J37" s="17"/>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B38" s="17"/>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
@@ -3588,7 +3215,7 @@
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
@@ -3600,7 +3227,7 @@
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B40" s="17"/>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -3612,7 +3239,7 @@
       <c r="J40" s="17"/>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -3624,7 +3251,7 @@
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
       <c r="D42" s="17"/>
@@ -3636,7 +3263,7 @@
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -3648,7 +3275,7 @@
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
       <c r="D44" s="17"/>
@@ -3660,7 +3287,7 @@
       <c r="J44" s="17"/>
       <c r="K44" s="17"/>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B45" s="17"/>
       <c r="C45" s="17"/>
       <c r="D45" s="17"/>
@@ -3672,7 +3299,7 @@
       <c r="J45" s="17"/>
       <c r="K45" s="17"/>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B46" s="17"/>
       <c r="C46" s="17"/>
       <c r="D46" s="17"/>
@@ -3684,7 +3311,7 @@
       <c r="J46" s="17"/>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -3696,7 +3323,7 @@
       <c r="J47" s="17"/>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B48" s="17"/>
       <c r="C48" s="17"/>
       <c r="D48" s="17"/>
@@ -3708,7 +3335,7 @@
       <c r="J48" s="17"/>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B49" s="17"/>
       <c r="C49" s="17"/>
       <c r="D49" s="17"/>
@@ -3728,9 +3355,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C80FB96-22CB-4B43-9A87-9AB2DFEB458D}">
   <dimension ref="A1:AH49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B1" s="12" t="s">
         <v>20</v>
       </c>
@@ -3762,36 +3389,36 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="H2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="J2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="K2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
@@ -3804,9 +3431,9 @@
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B3" s="1">
         <v>34</v>
@@ -3849,9 +3476,9 @@
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B4" s="1">
         <v>38</v>
@@ -3894,9 +3521,9 @@
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B5" s="1">
         <v>17.5</v>
@@ -3939,9 +3566,9 @@
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B6" s="1">
         <v>1.1176470588235294</v>
@@ -3984,9 +3611,9 @@
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B7" s="1">
         <v>0.51470588235294112</v>
@@ -4029,7 +3656,7 @@
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>0</v>
       </c>
@@ -4064,7 +3691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>1</v>
       </c>
@@ -4100,7 +3727,7 @@
       </c>
       <c r="L9" s="3"/>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>2</v>
       </c>
@@ -4136,7 +3763,7 @@
       </c>
       <c r="L10" s="3"/>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>3</v>
       </c>
@@ -4172,7 +3799,7 @@
       </c>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>4</v>
       </c>
@@ -4208,7 +3835,7 @@
       </c>
       <c r="L12" s="3"/>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>5</v>
       </c>
@@ -4255,7 +3882,7 @@
       <c r="AG13" s="1"/>
       <c r="AH13" s="1"/>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>6</v>
       </c>
@@ -4297,7 +3924,7 @@
       <c r="AB14" s="1"/>
       <c r="AC14" s="1"/>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>7</v>
       </c>
@@ -4339,7 +3966,7 @@
       <c r="AB15" s="1"/>
       <c r="AC15" s="1"/>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>8</v>
       </c>
@@ -4385,7 +4012,7 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>9</v>
       </c>
@@ -4421,7 +4048,7 @@
       </c>
       <c r="L17" s="3"/>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>10</v>
       </c>
@@ -4457,7 +4084,7 @@
       </c>
       <c r="L18" s="3"/>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>11</v>
       </c>
@@ -4493,7 +4120,7 @@
       </c>
       <c r="L19" s="3"/>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>12</v>
       </c>
@@ -4529,7 +4156,7 @@
       </c>
       <c r="L20" s="3"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>13</v>
       </c>
@@ -4564,7 +4191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>14</v>
       </c>
@@ -4599,7 +4226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>15</v>
       </c>
@@ -4634,7 +4261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>16</v>
       </c>
@@ -4669,7 +4296,7 @@
         <v>153.36904761904762</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>17</v>
       </c>
@@ -4704,7 +4331,7 @@
         <v>153.36904761904762</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>18</v>
       </c>
@@ -4745,7 +4372,7 @@
       <c r="AB26" s="1"/>
       <c r="AC26" s="1"/>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>19</v>
       </c>
@@ -4786,7 +4413,7 @@
       <c r="AB27" s="1"/>
       <c r="AC27" s="1"/>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.3">
       <c r="X28" s="3"/>
       <c r="Y28" s="5"/>
       <c r="Z28" s="5"/>
@@ -4794,7 +4421,7 @@
       <c r="AB28" s="1"/>
       <c r="AC28" s="1"/>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
       <c r="X29" s="3"/>
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
@@ -4802,7 +4429,7 @@
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
@@ -4820,7 +4447,7 @@
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -4832,7 +4459,7 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -4844,7 +4471,7 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -4856,7 +4483,7 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -4868,7 +4495,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -4880,7 +4507,7 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -4892,7 +4519,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -4904,7 +4531,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -4916,7 +4543,7 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -4928,7 +4555,7 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -4940,7 +4567,7 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -4952,7 +4579,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
@@ -4964,7 +4591,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -4976,7 +4603,7 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -4988,7 +4615,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
@@ -5000,7 +4627,7 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
@@ -5012,7 +4639,7 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
       <c r="D47" s="8"/>
@@ -5024,7 +4651,7 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
@@ -5036,7 +4663,7 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>

</xml_diff>